<commit_message>
add matches, gaps, reasoning to tracker. duplicate detection of urls. 70% threshold for decision apply or skip
</commit_message>
<xml_diff>
--- a/tracker.xlsx
+++ b/tracker.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G4"/>
+  <dimension ref="A1:J2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -444,10 +444,25 @@
       </c>
       <c r="F1" t="inlineStr">
         <is>
+          <t>Matches</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Gaps</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Reasoning</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
           <t>URL</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
@@ -479,80 +494,25 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
+          <t>Python development, API integrations, Cross-functional collaboration, Problem solving</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Low-code tools (Zapier), Europe residency requirement</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>You have strong technical skills in Python and JavaScript, experience with API integrations, and a proven ability to collaborate cross-functionally and solve complex technical problems. Your background in data-driven problem solving fits well with the role's requirements to build and automate solutions that streamline operations. However, knowledge of low-code tools such as Zapier is not evident. Despite being based in Stockholm, Sweden, you are within Europe which satisfies the location requirement. Given these factors, you are a strong fit for the role and should apply.</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
           <t>https://careers.hostaway.com/o/internal-ai-tools-specialist-remote-europe?source=LinkedIn</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>2026-04-16</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Saab</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>EU Project &amp; Consortium Coordinator</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Defence and Security</t>
-        </is>
-      </c>
-      <c r="D3" t="n">
-        <v>70</v>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>apply</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>https://www.saab.com/career/job-opportunities/eu-project--consortium-coordinator?source_board=LinkedIn</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>2026-04-16</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Imperial Brands</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Unspecified</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Tobacco</t>
-        </is>
-      </c>
-      <c r="D4" t="n">
-        <v>65</v>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>apply</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>https://imperialbrands.recruitmentplatform.com/AAACbwAA-e5f0a242-dfb0-469d-8544-e3333922abc5/apply.html?jobId=PU7FK026203F3VBQB8N7V79IR-36308&amp;langCode=en_GB&amp;board_id=107477&amp;source_board=LinkedIn_Slots</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
+      <c r="J2" t="inlineStr">
         <is>
           <t>2026-04-16</t>
         </is>

</xml_diff>

<commit_message>
fix tracker indentation bug, consistent decision threshold in output files, clean outputs on each run
</commit_message>
<xml_diff>
--- a/tracker.xlsx
+++ b/tracker.xlsx
@@ -481,11 +481,11 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Vacation Rental Management</t>
+          <t>Technology/Vacation Rental Management</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>85</v>
+        <v>75</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -494,17 +494,17 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Python development, API integrations, Cross-functional collaboration, Problem solving</t>
+          <t>Python, JavaScript, API Integrations, Problem Solving, Cross-functional collaboration</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Low-code tools (Zapier), Europe residency requirement</t>
+          <t>Zapier, Low-code tools experience</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>You have strong technical skills in Python and JavaScript, experience with API integrations, and a proven ability to collaborate cross-functionally and solve complex technical problems. Your background in data-driven problem solving fits well with the role's requirements to build and automate solutions that streamline operations. However, knowledge of low-code tools such as Zapier is not evident. Despite being based in Stockholm, Sweden, you are within Europe which satisfies the location requirement. Given these factors, you are a strong fit for the role and should apply.</t>
+          <t>You have strong programming skills in Python and JavaScript, a solid understanding of API operations, and experience in cross-functional environments, which align well with the requirements of the job at Hostaway. Your analytical background and problem-solving skills are also a fit. However, your experience with low-code tools like Zapier is not directly mentioned, which could be a gap considering their specific usage in the role. Despite this, your skill set is strong enough to suggest applying.</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">

</xml_diff>

<commit_message>
add CV recommendations to output and tracker
</commit_message>
<xml_diff>
--- a/tracker.xlsx
+++ b/tracker.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J2"/>
+  <dimension ref="A1:L2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -459,10 +459,20 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
+          <t>CV: Add</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>CV: Remove</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
           <t>URL</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
@@ -481,7 +491,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Technology/Vacation Rental Management</t>
+          <t>Vacation Rental Management</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -494,25 +504,31 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Python, JavaScript, API Integrations, Problem Solving, Cross-functional collaboration</t>
+          <t>Python/JS, AI agents, API integrations, Automation, Technical problem solving</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Zapier, Low-code tools experience</t>
+          <t>Low-code tools (Zapier), Business operations experience</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>You have strong programming skills in Python and JavaScript, a solid understanding of API operations, and experience in cross-functional environments, which align well with the requirements of the job at Hostaway. Your analytical background and problem-solving skills are also a fit. However, your experience with low-code tools like Zapier is not directly mentioned, which could be a gap considering their specific usage in the role. Despite this, your skill set is strong enough to suggest applying.</t>
+          <t>You have a strong background in Python, JavaScript, and API integrations, which aligns well with the technical requirements of designing AI tools and automating workflows. Your ability to problem-solve and work with data models complements the role's focus on efficiency and value creation. However, experience with low-code tools like Zapier and deeper business operations exposure are limited, slightly impacting the fit score.</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
+          <t>Experience with low-code tools, Business operations focus</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr">
+        <is>
           <t>https://careers.hostaway.com/o/internal-ai-tools-specialist-remote-europe?source=LinkedIn</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr">
+      <c r="L2" t="inlineStr">
         <is>
           <t>2026-04-16</t>
         </is>

</xml_diff>

<commit_message>
fix tracker indentation, add temperature=0 for consistent scoring
</commit_message>
<xml_diff>
--- a/tracker.xlsx
+++ b/tracker.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L2"/>
+  <dimension ref="A1:L3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -481,54 +481,114 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Hostaway</t>
+          <t>MPower Plus</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Internal AI Tools Specialist</t>
+          <t>Business Analyst</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Vacation Rental Management</t>
+          <t>IT Services and Consulting</t>
         </is>
       </c>
       <c r="D2" t="n">
+        <v>70</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>apply</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Agile practices, Stakeholder collaboration, Domain analysis</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Nordic P&amp;C insurance, User stories</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>You have a strong background in Agile methodologies, stakeholder collaboration, and domain analysis, which aligns well with the job's requirements. However, you lack specific experience with Nordic P&amp;C insurance processes and developing detailed user stories. Despite these gaps, your overall tech-business bridge and experience in similar roles make you a strong candidate.</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Nordic P&amp;C insurance familiarity, User story examples</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>Focus on linguistics projects</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/4399243835/?alternateChannel=search&amp;eBP=CwEAAAGdloZUmJIfKH6BYfGjnJs3oMBy7rrewb_nxPR4w4NETc4zOzxPDRT95WRBtNcUmj_kSafjhdG6yAfrU86d2N3Sp0i36_j4JgN9oov0z53QMIU4HjzRiI5CnmHwfLl3UmxhkW7v8XKfb1CHLzgzl-z_VNgCqak8ZHci8NFlCw_De1a84SIKuJMj915a_DYCyEdpKCqMpFuwI1bZJTV2RONW_LAVqgGRThb-LIm1WBwsqOxxRvBrm4eL8P7rDype3v_w-6IiwQOeIRklqTmgIHDyoYFlwuNmDAPmxQIWaAEQULNjAU0VGd8NaZaxAdOt4svMoOQiDDlrdAX5wPjqdjxRmC7nAia7Ap2BNXiMlpTIljGLE5oJGQe69w46K6jOIweCDsnpL-XsD9ZGvzmjQngHm5hKud0o5Rk2oVceBrh2d74UGfEtcKGYoidIzFQQjrfJnjKX3CZMTtS570Hv9IEmDWOdwUbcdtCbbuXasys-&amp;trk=d_flagship3_jobs_discovery_jymbii&amp;refId=P0egXggO2KFWmocsR%2BGkTg%3D%3D&amp;trackingId=iy5q5FwxufyuFigWtSR98g%3D%3D</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>emagine</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Data Visualization &amp; Analytics Contractor – Cost Engineering (FinOps)</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Technology Consulting</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
         <v>75</v>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="E3" t="inlineStr">
         <is>
           <t>apply</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>Python/JS, AI agents, API integrations, Automation, Technical problem solving</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>Low-code tools (Zapier), Business operations experience</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>You have a strong background in Python, JavaScript, and API integrations, which aligns well with the technical requirements of designing AI tools and automating workflows. Your ability to problem-solve and work with data models complements the role's focus on efficiency and value creation. However, experience with low-code tools like Zapier and deeper business operations exposure are limited, slightly impacting the fit score.</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>Experience with low-code tools, Business operations focus</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>https://careers.hostaway.com/o/internal-ai-tools-specialist-remote-europe?source=LinkedIn</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr">
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Python, Data modeling, Azure DevOps, Scrum/Agile</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Power BI, Professional SQL experience</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>You have a strong foundation in data modeling, Python development, and experience in agile environments, which aligns well with the job's requirements. However, your lack of professional experience using Power BI and SQL could be a drawback for this role, which may demand these skills for data visualization and analytics tasks.</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Power BI projects, SQL projects</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>https://portal.emagine.org/jobs/175762/data-visualization-analytics-contractor-cost-engineering-finops?utm_source=LinkedIn</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
         <is>
           <t>2026-04-16</t>
         </is>

</xml_diff>